<commit_message>
feat: import affiliate schools (2026-09-08)
</commit_message>
<xml_diff>
--- a/data/a8-import/アフィリエイト案件_スキルアップ図鑑.xlsx
+++ b/data/a8-import/アフィリエイト案件_スキルアップ図鑑.xlsx
@@ -126,10 +126,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -161,10 +161,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>

</xml_diff>